<commit_message>
fix my cart quantity change updating and fix revenue page
</commit_message>
<xml_diff>
--- a/swd392/document/dataset/Nutrients.xlsx
+++ b/swd392/document/dataset/Nutrients.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Id</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>Protein</t>
+  </si>
+  <si>
+    <t>cb91e0a9-3012-4217-91a1-30d4cb626895</t>
   </si>
   <si>
     <t>Carbs</t>
@@ -48,10 +51,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-* #,##0.00\ &quot;₫&quot;_-;\-* #,##0.00\ &quot;₫&quot;_-;_-* &quot;-&quot;??\ &quot;₫&quot;_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00\ &quot;₫&quot;_-;\-* #,##0.00\ &quot;₫&quot;_-;_-* &quot;-&quot;??\ &quot;₫&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -81,6 +84,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="Arial"/>
       <charset val="0"/>
@@ -88,14 +98,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -124,7 +127,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -140,7 +143,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -162,31 +173,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -200,14 +197,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
@@ -225,7 +228,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -252,13 +255,115 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -270,169 +375,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -569,6 +572,15 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
         <color theme="4"/>
       </bottom>
@@ -590,6 +602,41 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -605,41 +652,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -654,160 +666,151 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="15" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1236,10 +1239,10 @@
     </row>
     <row r="3" ht="22.5" customHeight="1" spans="1:22">
       <c r="A3" s="5" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1264,10 +1267,10 @@
     </row>
     <row r="4" ht="22.5" customHeight="1" spans="1:22">
       <c r="A4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -1292,10 +1295,10 @@
     </row>
     <row r="5" ht="22.5" customHeight="1" spans="1:22">
       <c r="A5" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>

</xml_diff>